<commit_message>
Remove temporary Matrix_DevelopmentLog file and update cycle configuration to use demo CSV. Adjust plugin selection order for clarity.
</commit_message>
<xml_diff>
--- a/Matrix_DevelopmentLog.xlsx
+++ b/Matrix_DevelopmentLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Python\Matrix_v2_retry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5314AE5-9685-46AC-A03C-218809DBAE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8254291F-9D49-4391-A4D0-BB55CA72C3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{879C8776-A109-45EF-BC97-4BD35C18C0CA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="145">
   <si>
     <t>Item #</t>
   </si>
@@ -443,6 +443,45 @@
   </si>
   <si>
     <t xml:space="preserve">5/18/2026 - confirmed unlock is ok, ecm stays unlocked if not powered down (desktop setup) so once unlocked once, the 'key' in the config stops mattering until its powered down.  </t>
+  </si>
+  <si>
+    <t>Add units to custom channel generation</t>
+  </si>
+  <si>
+    <t>Add Device Type Column to Configuration Dialog</t>
+  </si>
+  <si>
+    <t>Udpate</t>
+  </si>
+  <si>
+    <t>Reduce cycle telemetry in 'System' section of table</t>
+  </si>
+  <si>
+    <t>CAN discovery seems a little bugged out, sometimes defaults to bank entry even though I picked CAN1 or CAN2 previously.</t>
+  </si>
+  <si>
+    <t>Cycle Control UI did not refresh when I loaded in new cycle</t>
+  </si>
+  <si>
+    <t>App</t>
+  </si>
+  <si>
+    <t>Post Test Comments</t>
+  </si>
+  <si>
+    <t>Plugins do not resize when shrinking dialog window</t>
+  </si>
+  <si>
+    <t>LoadBank</t>
+  </si>
+  <si>
+    <t>Take Control Button doesn't work anymore after 'heartbeat' update for 700kw, take control is false but load can still be applied.</t>
+  </si>
+  <si>
+    <t>Load Setpoint should be integer intput, no decimals</t>
+  </si>
+  <si>
+    <t>Needs to be more generic, currently only applies to load control, but cycles have been used for multiple signals and triggered off other channels (volts out, trigger on ignition or RPM etc)</t>
   </si>
 </sst>
 </file>
@@ -857,8 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -897,7 +935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -918,7 +956,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -939,7 +977,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -960,7 +998,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1025,7 +1063,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1048,7 +1086,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1071,7 +1109,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1094,7 +1132,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1113,7 +1151,7 @@
       </c>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1132,7 +1170,7 @@
       </c>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1155,7 +1193,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1174,7 +1212,7 @@
       </c>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1243,7 +1281,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1262,7 +1300,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1283,7 +1321,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1306,7 +1344,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1327,7 +1365,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1350,7 +1388,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1371,7 +1409,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1394,7 +1432,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1413,7 +1451,7 @@
       </c>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1434,7 +1472,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -1454,7 +1492,7 @@
       <c r="G27" s="3"/>
       <c r="M27" s="8"/>
     </row>
-    <row r="28" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -1473,7 +1511,7 @@
       </c>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -1494,7 +1532,7 @@
       </c>
       <c r="G29" s="3"/>
     </row>
-    <row r="30" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -1518,7 +1556,7 @@
       </c>
       <c r="L30" s="7"/>
     </row>
-    <row r="31" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -1537,7 +1575,7 @@
       </c>
       <c r="G31" s="3"/>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -1556,7 +1594,7 @@
       </c>
       <c r="G32" s="3"/>
     </row>
-    <row r="33" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -1579,7 +1617,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>32</v>
       </c>
@@ -1600,7 +1638,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>33</v>
       </c>
@@ -1619,7 +1657,7 @@
       </c>
       <c r="G35" s="3"/>
     </row>
-    <row r="36" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>34</v>
       </c>
@@ -1640,7 +1678,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>35</v>
       </c>
@@ -1663,7 +1701,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>36</v>
       </c>
@@ -1682,7 +1720,7 @@
       </c>
       <c r="G38" s="3"/>
     </row>
-    <row r="39" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>37</v>
       </c>
@@ -1701,7 +1739,7 @@
       </c>
       <c r="G39" s="3"/>
     </row>
-    <row r="40" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>38</v>
       </c>
@@ -1724,7 +1762,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>39</v>
       </c>
@@ -1743,7 +1781,7 @@
       </c>
       <c r="G41" s="3"/>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>40</v>
       </c>
@@ -1764,7 +1802,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>41</v>
       </c>
@@ -1783,7 +1821,7 @@
       </c>
       <c r="G43" s="3"/>
     </row>
-    <row r="44" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>42</v>
       </c>
@@ -1806,7 +1844,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>43</v>
       </c>
@@ -1825,7 +1863,7 @@
       </c>
       <c r="G45" s="3"/>
     </row>
-    <row r="46" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>43</v>
       </c>
@@ -1844,7 +1882,7 @@
       </c>
       <c r="G46" s="3"/>
     </row>
-    <row r="47" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>44</v>
       </c>
@@ -1867,7 +1905,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>45</v>
       </c>
@@ -1890,7 +1928,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>46</v>
       </c>
@@ -1934,7 +1972,7 @@
       </c>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>48</v>
       </c>
@@ -1953,7 +1991,7 @@
       </c>
       <c r="G51" s="3"/>
     </row>
-    <row r="52" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>49</v>
       </c>
@@ -1974,7 +2012,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -2018,7 +2056,7 @@
       </c>
       <c r="G54" s="3"/>
     </row>
-    <row r="55" spans="1:7" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -2041,7 +2079,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -2060,7 +2098,7 @@
       </c>
       <c r="G56" s="3"/>
     </row>
-    <row r="57" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -2083,7 +2121,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -2102,7 +2140,7 @@
       </c>
       <c r="G58" s="3"/>
     </row>
-    <row r="59" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -2146,7 +2184,7 @@
       </c>
       <c r="G60" s="3"/>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -2165,7 +2203,7 @@
       </c>
       <c r="G61" s="3"/>
     </row>
-    <row r="62" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -2179,22 +2217,207 @@
         <v>128</v>
       </c>
       <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
+      <c r="F62" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="G62" s="3"/>
     </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>60</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G63" s="3"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>61</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G64" s="3"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <v>62</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G65" s="3"/>
+    </row>
+    <row r="66" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <v>63</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G66" s="3"/>
+    </row>
+    <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <v>64</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>65</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="3"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
+        <v>66</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <v>67</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
+        <v>68</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
+        <v>69</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G72" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G62" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Yes"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="6">
-      <filters blank="1">
-        <filter val="IN PROCESS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G62" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Cycle plugin documentation and configuration
- Refreshed Cycle plugin documentation to clarify output mapping and CSV structure.
- Updated cycle configuration to support new output types and improved usability.
- Enhanced integration details with LoadBank and NI DAQ for better state management during cycles.
- Adjusted README and changelog to reflect recent changes and improvements.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Matrix_DevelopmentLog.xlsx
+++ b/Matrix_DevelopmentLog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Python\Matrix_v2_retry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8254291F-9D49-4391-A4D0-BB55CA72C3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC683EB-EF50-4860-A84F-8FFB513A3FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{879C8776-A109-45EF-BC97-4BD35C18C0CA}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="146">
   <si>
     <t>Item #</t>
   </si>
@@ -434,10 +434,6 @@
     <t>Standalone tool to pick sqlite file (or folder) and export instead of waiting for end of test or if crash occurs</t>
   </si>
   <si>
-    <t>750kW complete
-5/14/2026 - Reviewed 1.5MW setup, should work as 750KW works and setup is very similar but still need to test.  700kW mapping yaml updated and UI updated for heartbeat monitoring.  Need to test</t>
-  </si>
-  <si>
     <t>5/4/2026 - single command line launch complete, release will be compiled exe
 5/14/2026 - exe with onedir setup (expect large).  Store in network drives for distribution, build locally, use git for source code, include readme with necessary installs outside of onedir included files.</t>
   </si>
@@ -482,6 +478,14 @@
   </si>
   <si>
     <t>Needs to be more generic, currently only applies to load control, but cycles have been used for multiple signals and triggered off other channels (volts out, trigger on ignition or RPM etc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">750kW complete
+5/14/2026 - Reviewed 1.5MW setup, should work as 750KW works and setup is very similar but still need to test.  700kW mapping yaml updated and UI updated for heartbeat monitoring.  Need to test
+5/20/2026 - 1.5MW tested and commands work.  </t>
+  </si>
+  <si>
+    <t>5/22/2026 - Update complete, need to test live with engine to confirm functionality</t>
   </si>
 </sst>
 </file>
@@ -896,6 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -935,7 +940,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -956,7 +961,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -977,7 +982,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -998,7 +1003,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1040,7 +1045,7 @@
       </c>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1054,7 +1059,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>70</v>
@@ -1063,7 +1068,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1086,7 +1091,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1109,7 +1114,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1132,7 +1137,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1151,7 +1156,7 @@
       </c>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1170,7 +1175,7 @@
       </c>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1193,7 +1198,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1212,7 +1217,7 @@
       </c>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1272,7 +1277,7 @@
         <v>35</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>70</v>
@@ -1281,7 +1286,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1300,7 +1305,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1321,7 +1326,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1344,7 +1349,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1365,7 +1370,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1388,7 +1393,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1409,7 +1414,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1432,7 +1437,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1451,7 +1456,7 @@
       </c>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1472,7 +1477,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -1492,7 +1497,7 @@
       <c r="G27" s="3"/>
       <c r="M27" s="8"/>
     </row>
-    <row r="28" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -1511,7 +1516,7 @@
       </c>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -1532,7 +1537,7 @@
       </c>
       <c r="G29" s="3"/>
     </row>
-    <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -1556,7 +1561,7 @@
       </c>
       <c r="L30" s="7"/>
     </row>
-    <row r="31" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -1575,7 +1580,7 @@
       </c>
       <c r="G31" s="3"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -1594,7 +1599,7 @@
       </c>
       <c r="G32" s="3"/>
     </row>
-    <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -1617,7 +1622,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>32</v>
       </c>
@@ -1638,7 +1643,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>33</v>
       </c>
@@ -1657,7 +1662,7 @@
       </c>
       <c r="G35" s="3"/>
     </row>
-    <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>34</v>
       </c>
@@ -1678,7 +1683,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>35</v>
       </c>
@@ -1701,7 +1706,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>36</v>
       </c>
@@ -1720,7 +1725,7 @@
       </c>
       <c r="G38" s="3"/>
     </row>
-    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>37</v>
       </c>
@@ -1739,7 +1744,7 @@
       </c>
       <c r="G39" s="3"/>
     </row>
-    <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>38</v>
       </c>
@@ -1762,7 +1767,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>39</v>
       </c>
@@ -1781,7 +1786,7 @@
       </c>
       <c r="G41" s="3"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>40</v>
       </c>
@@ -1802,7 +1807,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>41</v>
       </c>
@@ -1821,7 +1826,7 @@
       </c>
       <c r="G43" s="3"/>
     </row>
-    <row r="44" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>42</v>
       </c>
@@ -1844,7 +1849,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>43</v>
       </c>
@@ -1863,7 +1868,7 @@
       </c>
       <c r="G45" s="3"/>
     </row>
-    <row r="46" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>43</v>
       </c>
@@ -1882,7 +1887,7 @@
       </c>
       <c r="G46" s="3"/>
     </row>
-    <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>44</v>
       </c>
@@ -1905,7 +1910,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>45</v>
       </c>
@@ -1928,7 +1933,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>46</v>
       </c>
@@ -1972,7 +1977,7 @@
       </c>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>48</v>
       </c>
@@ -1991,7 +1996,7 @@
       </c>
       <c r="G51" s="3"/>
     </row>
-    <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>49</v>
       </c>
@@ -2012,7 +2017,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -2054,9 +2059,11 @@
       <c r="F54" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G54" s="3"/>
-    </row>
-    <row r="55" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="G54" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -2079,7 +2086,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -2098,7 +2105,7 @@
       </c>
       <c r="G56" s="3"/>
     </row>
-    <row r="57" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -2121,7 +2128,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -2140,7 +2147,7 @@
       </c>
       <c r="G58" s="3"/>
     </row>
-    <row r="59" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -2177,14 +2184,16 @@
         <v>123</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G60" s="3"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G60" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -2203,7 +2212,7 @@
       </c>
       <c r="G61" s="3"/>
     </row>
-    <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -2233,7 +2242,7 @@
         <v>56</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E63" s="4"/>
       <c r="F63" s="4" t="s">
@@ -2241,7 +2250,7 @@
       </c>
       <c r="G63" s="3"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>61</v>
       </c>
@@ -2252,7 +2261,7 @@
         <v>56</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E64" s="4"/>
       <c r="F64" s="4" t="s">
@@ -2268,10 +2277,10 @@
         <v>93</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D65" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="E65" s="4"/>
       <c r="F65" s="4" t="s">
@@ -2279,7 +2288,7 @@
       </c>
       <c r="G65" s="3"/>
     </row>
-    <row r="66" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>63</v>
       </c>
@@ -2290,7 +2299,7 @@
         <v>14</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E66" s="4"/>
       <c r="F66" s="4" t="s">
@@ -2298,7 +2307,7 @@
       </c>
       <c r="G66" s="3"/>
     </row>
-    <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>64</v>
       </c>
@@ -2309,7 +2318,7 @@
         <v>14</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E67" s="4"/>
       <c r="F67" s="4" t="s">
@@ -2319,24 +2328,24 @@
         <v>37</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>65</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="3"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>66</v>
       </c>
@@ -2347,7 +2356,7 @@
         <v>56</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E69" s="4"/>
       <c r="F69" s="4" t="s">
@@ -2357,18 +2366,18 @@
         <v>37</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>67</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
@@ -2376,7 +2385,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>68</v>
       </c>
@@ -2387,7 +2396,7 @@
         <v>56</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E71" s="4"/>
       <c r="F71" s="4" t="s">
@@ -2408,16 +2417,29 @@
         <v>56</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E72" s="4"/>
+        <v>143</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>145</v>
+      </c>
       <c r="F72" s="4" t="s">
         <v>70</v>
       </c>
       <c r="G72" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G62" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}"/>
+  <autoFilter ref="A1:G72" xr:uid="{E1A3A675-DBF4-4BE1-B087-EFEC69B11BE9}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="Yes"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="6">
+      <filters blank="1">
+        <filter val="IN PROCESS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>